<commit_message>
Add non-breaking white spaces to the end of a column header.
</commit_message>
<xml_diff>
--- a/data/dataLoading/excel/ExcelLoaderTest.xlsx
+++ b/data/dataLoading/excel/ExcelLoaderTest.xlsx
@@ -1,32 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10512"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
   <workbookPr date1904="1" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jeckels/labkey/server/testAutomation/data/dataLoading/excel/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/danduffek/labkey/trunk_bio/server/testAutomation/data/dataLoading/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DDB285B3-66E7-9345-9DBE-518FB5CF52D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADF19844-22AD-C14B-A3BB-0F2592C9113A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="19820" tabRatio="500" xr2:uid="{0F1B91F7-EC75-2346-8855-7E05D96605EB}"/>
+    <workbookView xWindow="-44800" yWindow="8440" windowWidth="34560" windowHeight="19820" tabRatio="500" xr2:uid="{0F1B91F7-EC75-2346-8855-7E05D96605EB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="125725"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
@@ -90,8 +79,8 @@
     <t>des,crip,tion</t>
   </si>
   <si>
-    <t>scan
-First</t>
+    <t xml:space="preserve">scan
+First    </t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Issue 51933: Add non-breaking white spaces to the end of a column header. (#2229)
Co-authored-by: labkey-danield <danield@labkey.com>
</commit_message>
<xml_diff>
--- a/data/dataLoading/excel/ExcelLoaderTest.xlsx
+++ b/data/dataLoading/excel/ExcelLoaderTest.xlsx
@@ -1,32 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10512"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
   <workbookPr date1904="1" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jeckels/labkey/server/testAutomation/data/dataLoading/excel/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/danduffek/labkey/trunk_bio/server/testAutomation/data/dataLoading/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DDB285B3-66E7-9345-9DBE-518FB5CF52D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADF19844-22AD-C14B-A3BB-0F2592C9113A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="19820" tabRatio="500" xr2:uid="{0F1B91F7-EC75-2346-8855-7E05D96605EB}"/>
+    <workbookView xWindow="-44800" yWindow="8440" windowWidth="34560" windowHeight="19820" tabRatio="500" xr2:uid="{0F1B91F7-EC75-2346-8855-7E05D96605EB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="125725"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
@@ -90,8 +79,8 @@
     <t>des,crip,tion</t>
   </si>
   <si>
-    <t>scan
-First</t>
+    <t xml:space="preserve">scan
+First    </t>
   </si>
 </sst>
 </file>

</xml_diff>